<commit_message>
Calm the book UI: blank missings, toolbar filters, clearer rituals.
Thin Fact chips and dash noise, bundle NAV/Compare/Flags/Confirm filters, alias Inbox/Vault, and refresh demo fixtures so Confirm and Flags have real rows.
</commit_message>
<xml_diff>
--- a/fixtures/mis/FIXTURE_ONLY/cava/FIXTURE_ONLY-cava-FY26-M1-M6-history.xlsx
+++ b/fixtures/mis/FIXTURE_ONLY/cava/FIXTURE_ONLY-cava-FY26-M1-M6-history.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>Metric</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Net revenue</t>
+  </si>
+  <si>
+    <t>Plan revenue</t>
   </si>
   <si>
     <t>Gross margin %</t>
@@ -438,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -492,22 +495,22 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>48</v>
+        <v>3.01</v>
       </c>
       <c r="C3">
-        <v>49</v>
+        <v>3.15</v>
       </c>
       <c r="D3">
-        <v>50</v>
+        <v>3.35</v>
       </c>
       <c r="E3">
-        <v>51</v>
+        <v>3.43</v>
       </c>
       <c r="F3">
-        <v>50</v>
+        <v>3.59</v>
       </c>
       <c r="G3">
-        <v>52</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -515,22 +518,22 @@
         <v>9</v>
       </c>
       <c r="B4">
-        <v>0.99</v>
+        <v>48</v>
       </c>
       <c r="C4">
-        <v>1.01</v>
+        <v>49</v>
       </c>
       <c r="D4">
-        <v>1.04</v>
+        <v>50</v>
       </c>
       <c r="E4">
-        <v>1.05</v>
+        <v>51</v>
       </c>
       <c r="F4">
-        <v>1.07</v>
+        <v>50</v>
       </c>
       <c r="G4">
-        <v>1.1</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -538,22 +541,22 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>0.39</v>
+        <v>0.99</v>
       </c>
       <c r="C5">
-        <v>0.46</v>
+        <v>1.01</v>
       </c>
       <c r="D5">
-        <v>0.55</v>
+        <v>1.04</v>
       </c>
       <c r="E5">
-        <v>0.62</v>
+        <v>1.05</v>
       </c>
       <c r="F5">
-        <v>0.64</v>
+        <v>1.07</v>
       </c>
       <c r="G5">
-        <v>0.79</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -561,22 +564,22 @@
         <v>11</v>
       </c>
       <c r="B6">
-        <v>4.03</v>
+        <v>0.39</v>
       </c>
       <c r="C6">
-        <v>3.85</v>
+        <v>0.46</v>
       </c>
       <c r="D6">
-        <v>3.75</v>
+        <v>0.55</v>
       </c>
       <c r="E6">
-        <v>3.53</v>
+        <v>0.62</v>
       </c>
       <c r="F6">
-        <v>3.37</v>
+        <v>0.64</v>
       </c>
       <c r="G6">
-        <v>3.26</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -584,22 +587,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>0.32</v>
+        <v>4.03</v>
       </c>
       <c r="C7">
-        <v>0.31</v>
+        <v>3.85</v>
       </c>
       <c r="D7">
-        <v>0.32</v>
+        <v>3.75</v>
       </c>
       <c r="E7">
-        <v>0.3</v>
+        <v>3.53</v>
       </c>
       <c r="F7">
-        <v>0.29</v>
+        <v>3.37</v>
       </c>
       <c r="G7">
-        <v>0.3</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -607,22 +610,22 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>46</v>
+        <v>0.32</v>
       </c>
       <c r="C8">
-        <v>47</v>
+        <v>0.31</v>
       </c>
       <c r="D8">
-        <v>48</v>
+        <v>0.32</v>
       </c>
       <c r="E8">
-        <v>49</v>
+        <v>0.3</v>
       </c>
       <c r="F8">
-        <v>50</v>
+        <v>0.29</v>
       </c>
       <c r="G8">
-        <v>51</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -630,45 +633,68 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>23249</v>
+        <v>46</v>
       </c>
       <c r="C9">
-        <v>23947</v>
+        <v>47</v>
       </c>
       <c r="D9">
-        <v>24912</v>
+        <v>48</v>
       </c>
       <c r="E9">
-        <v>25402</v>
+        <v>49</v>
       </c>
       <c r="F9">
-        <v>26165</v>
+        <v>50</v>
       </c>
       <c r="G9">
-        <v>27219</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10">
+        <v>23249</v>
+      </c>
+      <c r="C10">
+        <v>23947</v>
+      </c>
+      <c r="D10">
+        <v>24912</v>
+      </c>
+      <c r="E10">
+        <v>25402</v>
+      </c>
+      <c r="F10">
+        <v>26165</v>
+      </c>
+      <c r="G10">
+        <v>27219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>16</v>
       </c>
-      <c r="C10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" t="s">
-        <v>16</v>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Spread fixture runways from ~2 to ~34 months so Command charts are not a flat cluster.
Closing cash now follows cash ÷ last-3-burn, and extract proposes null for an explicit dash so missing cash can be confirmed.
</commit_message>
<xml_diff>
--- a/fixtures/mis/FIXTURE_ONLY/cava/FIXTURE_ONLY-cava-FY26-M1-M6-history.xlsx
+++ b/fixtures/mis/FIXTURE_ONLY/cava/FIXTURE_ONLY-cava-FY26-M1-M6-history.xlsx
@@ -587,22 +587,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>4.03</v>
+        <v>4.8</v>
       </c>
       <c r="C7">
-        <v>3.85</v>
+        <v>4.67</v>
       </c>
       <c r="D7">
-        <v>3.75</v>
+        <v>4.55</v>
       </c>
       <c r="E7">
-        <v>3.53</v>
+        <v>4.42</v>
       </c>
       <c r="F7">
-        <v>3.37</v>
+        <v>4.29</v>
       </c>
       <c r="G7">
-        <v>3.26</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -610,22 +610,22 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="C8">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="D8">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="E8">
-        <v>0.3</v>
+        <v>0.36</v>
       </c>
       <c r="F8">
-        <v>0.29</v>
+        <v>0.37</v>
       </c>
       <c r="G8">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>